<commit_message>
Übersetzungsvorlage: Feste-Seiten-Texte aus dem Live-Stand (statt Blueprints)
Die Elementor-Seiten wurden live redaktionell weiterentwickelt – die
Vorlage übersetzt jetzt den tatsächlichen Stand; Referenzen zeigen auf
Seite:Widget-ID:Feld für das maschinelle Einpflegen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YHywkFmV2Tg5zSx1wJDo3Z
</commit_message>
<xml_diff>
--- a/docs/Uebersetzungsvorlage-Energiesozietaet-EN.xlsx
+++ b/docs/Uebersetzungsvorlage-Energiesozietaet-EN.xlsx
@@ -599,14 +599,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,18 +644,18 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Recht · Steuern · Beratung</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>home.title</t>
+          <t>live:home:956e323:title</t>
         </is>
       </c>
     </row>
@@ -672,13 +672,17 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Recht · Steuern · Beratung</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr"/>
+          <t>Expertise trifft &lt;span class="text-bg-green"&gt;Leidenschaft.&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Expertise meets &lt;span class="text-bg-green"&gt;passion.&lt;/span&gt;  ← BEISPIEL</t>
+        </is>
+      </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:home:a78add1:title</t>
         </is>
       </c>
     </row>
@@ -690,22 +694,18 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Expertise trifft &lt;span class="text-bg-green"&gt;Leidenschaft.&lt;/span&gt;</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Expertise meets &lt;span class="text-bg-green"&gt;passion.&lt;/span&gt;  ← BEISPIEL</t>
-        </is>
-      </c>
+          <t>&lt;p&gt;Wir sind ein &lt;em&gt;junges, innovatives Beratungsunternehmen&lt;/em&gt;, dessen langjährig erfahrene Rechtsanwälte, Steuer- und Unternehmensberater sich der &lt;em&gt;Transformation der öffentlichen Hand und der Energiewirtschaft&lt;/em&gt; verschrieben haben. Wir arbeiten hoch spezialisiert, fachübergreifend und fokussiert an den Themen unserer Zeit.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:home:9daf9b3:editor</t>
         </is>
       </c>
     </row>
@@ -717,18 +717,18 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir sind ein &lt;em&gt;junges, innovatives Beratungsunternehmen&lt;/em&gt;, dessen langjährig erfahrene Rechtsanwälte, Steuer- und Unternehmensberater sich der &lt;em&gt;Transformation der öffentlichen Hand und der Energiewirtschaft&lt;/em&gt; verschrieben haben. Wir arbeiten hoch spezialisiert, fachübergreifend und fokussiert an den Themen unserer Zeit.&lt;/p&gt;</t>
+          <t>Berufsträger &amp; Mitarbeiter</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.2.settings.editor</t>
+          <t>live:home:73e2b42:title</t>
         </is>
       </c>
     </row>
@@ -740,18 +740,18 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Leistungen entdecken →</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.3.settings.text</t>
+          <t>live:home:64e8eb7:title</t>
         </is>
       </c>
     </row>
@@ -763,18 +763,18 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Unser Team kennenlernen →</t>
+          <t>Gegründet</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.4.settings.text</t>
+          <t>live:home:019bba5:title</t>
         </is>
       </c>
     </row>
@@ -791,13 +791,13 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Berufsträger &amp; Mitarbeiter</t>
+          <t>Standorte · DUS · HH · MA</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.5.elements.0.elements.1.settings.title</t>
+          <t>live:home:2184912:title</t>
         </is>
       </c>
     </row>
@@ -814,13 +814,13 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Beratungsfelder</t>
+          <t>Unsere Philosophie</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.5.elements.1.elements.1.settings.title</t>
+          <t>live:home:c8e9935:title</t>
         </is>
       </c>
     </row>
@@ -837,13 +837,13 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Gegründet</t>
+          <t>Interdisziplinäre Beratung in komplexen Fragestellungen: &lt;span class="text-bg-green"&gt;fokussiert, ergebnisorientiert und kreativ.&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.5.elements.2.elements.1.settings.title</t>
+          <t>live:home:a86c7b2:title</t>
         </is>
       </c>
     </row>
@@ -855,18 +855,18 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Standorte · DUS · HH · MA</t>
+          <t>&lt;p&gt;Transformation ist eine Mammutaufgabe: dafür braucht es viele, das schafft niemand allein. Wir – das Team der Energiesozietät – verstehen uns als einer der vielen. Wir werden Teil sein und möchten Verantwortung übernehmen. Unser Ziel ist, Lösungen zu entwickeln für die überaus komplexen Transformationsfragen unserer Zeit. Wir unterstützen unsere Mandanten dabei, Rahmenbedingungen zu schaffen, Geschäftsmodelle zu entwickeln und Organisationen dafür zu verändern, dass sie die Herausforderungen der Zeit meistern.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.0.elements.0.elements.5.elements.3.elements.1.settings.title</t>
+          <t>live:home:bc2ceff:editor</t>
         </is>
       </c>
     </row>
@@ -878,18 +878,18 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Unser Anspruch</t>
+          <t>&lt;p&gt;&lt;a class="es-link" href="/philosophie/"&gt;Mehr erfahren&lt;/a&gt; · &lt;a class="es-link" href="/team/"&gt;Unser Team&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.1.elements.0.elements.0.settings.title</t>
+          <t>live:home:79ab413:editor</t>
         </is>
       </c>
     </row>
@@ -906,13 +906,13 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Hoch spezialisiert.&lt;br&gt;Fachübergreifend.&lt;br&gt;&lt;span class="text-bg-green"&gt;Ergebnisorientiert.&lt;/span&gt;</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.1.elements.0.elements.1.settings.title</t>
+          <t>live:home:a00189d:title</t>
         </is>
       </c>
     </row>
@@ -924,18 +924,18 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir arbeiten hoch spezialisiert, fachübergreifend und fokussiert an den Themen unserer Zeit — unaufgeregt, ergebnisorientiert und mit individuellen Persönlichkeiten.&lt;/p&gt;</t>
+          <t>Interdisziplinäre Beratung.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.1.elements.1.elements.0.settings.editor</t>
+          <t>live:home:26b2b9e:title</t>
         </is>
       </c>
     </row>
@@ -952,13 +952,13 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;a class="es-link" href="/philosophie/"&gt;Unsere Philosophie&lt;/a&gt; · &lt;a class="es-link" href="/team/"&gt;Unser Team&lt;/a&gt;&lt;/p&gt;</t>
+          <t>&lt;p&gt;Wir denken Lösungen vom Ende her: strategische, technische, betriebs- und finanzwirtschaftliche, juristische und steuerliche Lösungen stellen wir dafür in den Gesamtkontext.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.1.elements.1.elements.1.settings.editor</t>
+          <t>live:home:3f7b470:editor</t>
         </is>
       </c>
     </row>
@@ -975,13 +975,13 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:home:6e56cd0:title</t>
         </is>
       </c>
     </row>
@@ -993,18 +993,18 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Interdisziplinäre Beratung.&lt;br&gt;&lt;span style="color:#5A6577;"&gt;Drei Felder, ein Gedanke.&lt;/span&gt;</t>
+          <t>&lt;p&gt;Wir stellen juristische Lösungen in den Gesamtkontext.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:home:b305beb:editor</t>
         </is>
       </c>
     </row>
@@ -1021,13 +1021,13 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir denken Lösungen vom Ende her: strategische, betriebswirtschaftliche, juristische und steuerliche Themen stellen wir in den Gesamtkontext.&lt;/p&gt;</t>
+          <t>&lt;p&gt;&lt;a class="es-link" href="/rechtsberatung/"&gt;Mehr erfahren →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.2.elements.0.elements.2.settings.editor</t>
+          <t>live:home:721b29d:editor</t>
         </is>
       </c>
     </row>
@@ -1044,13 +1044,13 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.0.elements.1.settings.title</t>
+          <t>live:home:fe07376:title</t>
         </is>
       </c>
     </row>
@@ -1067,13 +1067,13 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Energierecht, Vergaberecht, Regulierung, M&amp;A, Gesellschaftsrecht. Wir stellen juristische Lösungen in den Gesamtkontext.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Fortlaufende Steuerberatung, Gestaltungsberatung oder herausfordernde Neustrukturierungen?&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.0.elements.2.settings.editor</t>
+          <t>live:home:800df08:editor</t>
         </is>
       </c>
     </row>
@@ -1085,18 +1085,18 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>&lt;p&gt;&lt;a class="es-link" href="/steuerberatung/"&gt;Mehr erfahren →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.1.elements.1.settings.title</t>
+          <t>live:home:27ddd2d:editor</t>
         </is>
       </c>
     </row>
@@ -1108,18 +1108,18 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Fortlaufende Steuerberatung, Gestaltungsberatung und herausfordernde Neustrukturierungen für Versorger und Kommunen.&lt;/p&gt;</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.1.elements.2.settings.editor</t>
+          <t>live:home:cc1b440:title</t>
         </is>
       </c>
     </row>
@@ -1131,18 +1131,18 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>&lt;p&gt;Wir navigieren Sie durch strategische, wirtschaftliche und finanzielle Fragestellungen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr"/>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.2.elements.1.settings.title</t>
+          <t>live:home:5c74899:editor</t>
         </is>
       </c>
     </row>
@@ -1159,13 +1159,13 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir navigieren Sie durch strategische, wirtschaftliche und finanzielle Fragestellungen der Transformation.&lt;/p&gt;</t>
+          <t>&lt;p&gt;&lt;a class="es-link" href="/unternehmensberatung/"&gt;Mehr erfahren →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr"/>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.3.elements.2.elements.2.settings.editor</t>
+          <t>live:home:5283161:editor</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       <c r="D25" s="5" t="inlineStr"/>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.4.elements.0.elements.0.settings.title</t>
+          <t>live:home:f7782cf:title</t>
         </is>
       </c>
     </row>
@@ -1205,13 +1205,13 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>„Wir wollen mit unserer langjährigen Beratungs- und Netzwerkerfahrung unsere Mandantschaft bei den anstehenden Transformationen begleiten — und mit den individuellen Persönlichkeiten unseres Teams Mehrwert bieten."</t>
+          <t>„Wir wollen mit unserer langjährigen Beratungs- und Netzwerkerfahrung unsere Mandantschaft bei den anstehenden Transformationen begleiten und mit den individuellen Persönlichkeiten unseres Teams Mehrwert bieten."</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr"/>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.4.elements.0.elements.1.settings.title</t>
+          <t>live:home:3ecf491:title</t>
         </is>
       </c>
     </row>
@@ -1223,18 +1223,18 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Aktuelles · Neu</t>
+          <t>&lt;p class="es-gf-quote__name"&gt;Prof. Dr. Sven-Joachim Otto&lt;/p&gt;&lt;p class="es-gf-quote__role"&gt;Partner&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.5.elements.0.elements.0.settings.title</t>
+          <t>live:home:280b930:editor</t>
         </is>
       </c>
     </row>
@@ -1251,59 +1251,59 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Fachbeiträge.</t>
+          <t>Aktuelles</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr"/>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>home.elementor.5.elements.0.elements.1.settings.title</t>
+          <t>live:home:cc91154:title</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Philosophie</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Philosophie</t>
+          <t>Neues aus der Energiebranche.</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr"/>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>philosophie.title</t>
+          <t>live:home:02d46db:title</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Philosophie</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Philosophie</t>
+          <t>&lt;p style="margin-top:32px;"&gt;&lt;a class="es-link" href="/news/"&gt;Alle Beiträge ansehen →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:home:381dbb7:editor</t>
         </is>
       </c>
     </row>
@@ -1320,13 +1320,13 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Transformation ist eine&lt;br&gt;&lt;span class="text-bg-green"&gt;Mammutaufgabe.&lt;/span&gt;</t>
+          <t>Unsere Philosophie</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:aedaec6:title</t>
         </is>
       </c>
     </row>
@@ -1338,18 +1338,18 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Dafür braucht es viele. Das schafft niemand allein. Wir — das Team der Energiesozietät — verstehen uns als einer der vielen.&lt;/p&gt;</t>
+          <t>Ergebnisse,&lt;br&gt;&lt;span class="text-bg-green"&gt;die weitertragen.&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.0.elements.0.elements.2.settings.editor</t>
+          <t>live:philosophie:85f81ed:title</t>
         </is>
       </c>
     </row>
@@ -1361,18 +1361,18 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Wie wir arbeiten</t>
+          <t>&lt;p&gt;Transformation ist eine Mammutaufgabe: dafür braucht es viele, das schafft niemand allein. Wir – das Team der Energiesozietät – verstehen uns als einer der vielen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr"/>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.1.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:d4fe36c:editor</t>
         </is>
       </c>
     </row>
@@ -1389,13 +1389,13 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Fokussiert.&lt;br&gt;Ergebnis&amp;shy;orientiert.&lt;br&gt;&lt;span class="text-bg-green"&gt;Kreativ.&lt;/span&gt;</t>
+          <t>Ihre Aufgabe</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr"/>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.1.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:2b199fc:title</t>
         </is>
       </c>
     </row>
@@ -1407,18 +1407,18 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir sind Experten. Wir arbeiten hoch spezialisiert. Wir entwickeln ganzheitliche Lösungen, die strategische, betriebs- und finanzwirtschaftliche, juristische sowie steuerliche Fragen immer im Gesamtkontext betrachten.&lt;/p&gt;</t>
+          <t>Wir wissen, wie komplex&lt;br&gt;&lt;span class="text-bg-green"&gt;Ihre Aufgabe ist.&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.1.elements.1.elements.0.settings.editor</t>
+          <t>live:philosophie:e5b2f04:title</t>
         </is>
       </c>
     </row>
@@ -1435,13 +1435,13 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Das erfordert interdisziplinäres Denken, langjährige Erfahrung und die Bereitschaft, neu zu denken — gerade dort, wo sich Energiemärkte, regulatorische Rahmen und politische Entscheidungsprozesse gleichzeitig verändern.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Entscheidungsträger und Gestalter in der öffentlichen Wirtschaft und der Energieversorgung bewegen sich in einem extrem komplexen Umfeld.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr"/>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.1.elements.1.elements.1.settings.editor</t>
+          <t>live:philosophie:4bff70f:editor</t>
         </is>
       </c>
     </row>
@@ -1453,18 +1453,18 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Fokussiert</t>
+          <t>&lt;p&gt;Wir sind uns dieser Einflussfaktoren sehr bewusst. Deshalb beziehen wir Sie in unsere Lösungen stets mit ein, so dass unsere Beratungsergebnisse bestmöglich Ihren gestalterischen oder unternehmerischen Zielen dienen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr"/>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:ff672d9:editor</t>
         </is>
       </c>
     </row>
@@ -1481,13 +1481,13 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Wir arbeiten hoch spezialisiert an den Themen unserer Zeit. Kein Bauchladen, sondern vertiefte Expertise dort, wo die Transformation entschieden wird.</t>
+          <t>&lt;p&gt;Wir denken unsere Projekte vom Ende her. Unsere Beratung endet nicht mit der Beantwortung Ihrer konkreten Fragestellung. Vielmehr beinhaltet sie, dass wir berücksichtigen, wie Sie mit dem Endprodukt unserer Beratung weiterarbeiten, und bezieht auch eine adressatengerechte Ergebnisdarstellung und -kommunikation mit ein.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr"/>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.0.elements.2.settings.editor</t>
+          <t>live:philosophie:087529e:editor</t>
         </is>
       </c>
     </row>
@@ -1504,13 +1504,13 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Ergebnisorientiert</t>
+          <t>Wachsende Aufgaben</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr"/>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.1.elements.1.settings.title</t>
+          <t>live:philosophie:7acee97:title</t>
         </is>
       </c>
     </row>
@@ -1522,18 +1522,18 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Wir denken Lösungen vom Ende her. Strategische, technische, betriebs- und finanzwirtschaftliche, juristische sowie steuerliche Lösungen stellen wir in den Gesamtkontext.</t>
+          <t>Steigende regulatorische Anforderungen</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr"/>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.1.elements.2.settings.editor</t>
+          <t>live:philosophie:6be8327:title</t>
         </is>
       </c>
     </row>
@@ -1550,13 +1550,13 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Kreativ</t>
+          <t>Komplexe Entscheidungsprozesse</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr"/>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.2.elements.1.settings.title</t>
+          <t>live:philosophie:75a598a:title</t>
         </is>
       </c>
     </row>
@@ -1568,18 +1568,18 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Neue Fragestellungen verlangen neue Antworten. Wir verbinden langjährige Erfahrung aus Big-Four-Gesellschaften, spezialisierten Kanzleien und der Industrie mit einem agilen, pragmatischen Arbeitsrahmen.</t>
+          <t>Multi-Stakeholder</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr"/>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.2.elements.2.elements.2.settings.editor</t>
+          <t>live:philosophie:7fff22a:title</t>
         </is>
       </c>
     </row>
@@ -1596,13 +1596,13 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>„Unsere Mandanten bewegen sich in einem &lt;span class="text-bg-green"&gt;hochkomplexen&lt;/span&gt; und &lt;span class="text-bg-green"&gt;sich kontinuierlich wandelnden&lt;/span&gt; Umfeld. In diesem Umfeld treffen sie Entscheidungen, die ihre Unternehmen und Kommunen über Jahrzehnte prägen werden."</t>
+          <t>Was uns besonders macht</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr"/>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.3.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:887740f:title</t>
         </is>
       </c>
     </row>
@@ -1614,18 +1614,18 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Unsere Überzeugung&lt;/p&gt;</t>
+          <t>Langjährige interdisziplinäre Beratungserfahrung, vielfach erprobt.</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr"/>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.3.elements.0.elements.1.settings.editor</t>
+          <t>live:philosophie:beb45b9:title</t>
         </is>
       </c>
     </row>
@@ -1637,18 +1637,18 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Interdisziplinär</t>
+          <t>&lt;p&gt;Die Teammitglieder der Energiesozietät haben in unzähligen Projekten Erfahrungen gesammelt. Jeder zeichnet sich durch besondere Fähigkeiten aus. Was uns in der Energiesozietät gemeinsam besonders macht:&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.4.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:aa398d1:editor</t>
         </is>
       </c>
     </row>
@@ -1665,13 +1665,13 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Ein Team aus vier Perspektiven.</t>
+          <t>„Unseren Mandanten ist eines gemein: Sie bewegen sich alle in einem &lt;span class="text-bg-green"&gt;hochkomplexen&lt;/span&gt; und &lt;span class="text-bg-green"&gt;sich kontinuierlich weiterentwickelnden&lt;/span&gt; Umfeld."</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr"/>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.4.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:1624588:title</t>
         </is>
       </c>
     </row>
@@ -1688,13 +1688,13 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Ingenieure, Kaufleute, Rechtsanwälte und Steuerberater erarbeiten mit unseren Mandanten ganzheitliche, tragfähige Lösungen als Grundlage für gut abgewogene Entscheidungen.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Unsere Überzeugung&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr"/>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.4.elements.0.elements.2.settings.editor</t>
+          <t>live:philosophie:5030a9a:editor</t>
         </is>
       </c>
     </row>
@@ -1711,13 +1711,13 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Ingenieure</t>
+          <t>Interdisziplinär</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr"/>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:6abbaa8:title</t>
         </is>
       </c>
     </row>
@@ -1729,18 +1729,18 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Technische Lösungen und Machbarkeit im Energiesystem.</t>
+          <t>Ein Team aus vier Perspektiven.</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr"/>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.0.elements.1.settings.editor</t>
+          <t>live:philosophie:1f9e904:title</t>
         </is>
       </c>
     </row>
@@ -1752,18 +1752,18 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Kaufleute</t>
+          <t>&lt;p&gt;Unser Team von Ingenieuren, Kaufleuten, Rechtsanwälten und Steuerberatern erarbeitet mit Ihnen ganzheitliche, tragfähige Lösungen als Grundlage für eine gut abgewogene Entscheidung.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr"/>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.1.elements.0.settings.title</t>
+          <t>live:philosophie:9489fb8:editor</t>
         </is>
       </c>
     </row>
@@ -1775,18 +1775,18 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Betriebs- und finanzwirtschaftliche Bewertung und Strukturierung.</t>
+          <t>Rechtsanwälte</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr"/>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.1.elements.1.settings.editor</t>
+          <t>live:philosophie:63c111e:title</t>
         </is>
       </c>
     </row>
@@ -1798,18 +1798,18 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Rechtsanwälte</t>
+          <t>&lt;p&gt;Juristische Gestaltung im regulatorischen Gesamtkontext.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr"/>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.2.elements.0.settings.title</t>
+          <t>live:philosophie:a22a24c:editor</t>
         </is>
       </c>
     </row>
@@ -1821,18 +1821,18 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Juristische Gestaltung im regulatorischen Gesamtkontext.</t>
+          <t>Steuerberater</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr"/>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.2.elements.1.settings.editor</t>
+          <t>live:philosophie:f0c1b07:title</t>
         </is>
       </c>
     </row>
@@ -1844,18 +1844,18 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Steuerberater</t>
+          <t>&lt;p&gt;Steuerliche Struktur, Compliance und Gestaltungsspielräume.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr"/>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.3.elements.0.settings.title</t>
+          <t>live:philosophie:b5c3061:editor</t>
         </is>
       </c>
     </row>
@@ -1867,18 +1867,18 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Steuerliche Struktur, Compliance und Gestaltungsspielräume.</t>
+          <t>Wirtschaftsingenieure</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr"/>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.5.elements.3.elements.1.settings.editor</t>
+          <t>live:philosophie:b4428d6:title</t>
         </is>
       </c>
     </row>
@@ -1890,18 +1890,18 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Mandantschaft</t>
+          <t>&lt;p&gt;Technische Lösungen und Machbarkeit im Energiesystem.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr"/>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.6.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:e0c6f49:editor</t>
         </is>
       </c>
     </row>
@@ -1918,13 +1918,13 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Wen wir beraten.</t>
+          <t>Kaufleute</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr"/>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.6.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:7d68c2e:title</t>
         </is>
       </c>
     </row>
@@ -1941,13 +1941,13 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Mit unserem Beratungsangebot adressieren wir Energieversorgungsunternehmen, Bund, Länder und Kommunen sowie deren Einrichtungen und Unternehmen. Hinzu kommen private und öffentliche Infrastrukturdienstleister und Investoren.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Betriebs- und finanzwirtschaftliche Bewertung und Strukturierung.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr"/>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.6.elements.1.elements.0.settings.editor</t>
+          <t>live:philosophie:dedb25c:editor</t>
         </is>
       </c>
     </row>
@@ -1964,13 +1964,13 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Politikberatung</t>
+          <t>Mandantschaft</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr"/>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.7.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:b1e7ff8:title</t>
         </is>
       </c>
     </row>
@@ -1987,13 +1987,13 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Lösungen, die im&lt;br&gt;politischen Prozess&lt;br&gt;&lt;span class="text-bg-green"&gt;Akzeptanz finden.&lt;/span&gt;</t>
+          <t>Wen wir beraten.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr"/>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.7.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:77e5d39:title</t>
         </is>
       </c>
     </row>
@@ -2010,13 +2010,13 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir haben ein ausgeprägtes Verständnis von Energiemärkten, Verwaltungsorganisationen und ihren politischen Entscheidungsprozessen. Politikberatung ist integraler Bestandteil unserer Tätigkeit, um die Projekte unserer Mandanten zum Erfolg zu führen.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Mit unserem Beratungsangebot adressieren wir Energieversorgungsunternehmen, Bund, Länder und Kommunen sowie deren Einrichtungen und Unternehmen. Hinzu kommen private und öffentliche Infrastrukturdienstleister und Investoren.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr"/>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.7.elements.1.elements.0.settings.editor</t>
+          <t>live:philosophie:fd17733:editor</t>
         </is>
       </c>
     </row>
@@ -2028,87 +2028,87 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir entwickeln Konzepte für die Kommunikation von Lösungen im politischen Entscheidungsprozess — mit dem Ziel, bestmögliche Lösungen zu präsentieren, die eine breite Akzeptanz finden.&lt;/p&gt;</t>
+          <t>Politikberatung</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr"/>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>philosophie.elementor.7.elements.1.elements.1.settings.editor</t>
+          <t>live:philosophie:d37d8b6:title</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>Philosophie</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>Lösungen, die im&lt;br&gt;politischen Prozess&lt;br&gt;&lt;span class="text-bg-green"&gt;Akzeptanz finden.&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr"/>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>leistungen.title</t>
+          <t>live:philosophie:517955f:title</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>Philosophie</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>&lt;p&gt;Wir haben ein ausgeprägtes Verständnis von Energiemärkten, Verwaltungsorganisationen und ihren politischen Entscheidungsprozessen. Politikberatung ist integraler Bestandteil unserer Tätigkeit, um die Projekte unserer Mandanten zum Erfolg zu führen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr"/>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:philosophie:71f9031:editor</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Leistungen</t>
+          <t>Philosophie</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Interdisziplinäre&lt;br&gt;&lt;span class="text-bg-green"&gt;Beratung.&lt;/span&gt;</t>
+          <t>&lt;p&gt;Wir entwickeln für Sie Konzepte für die Kommunikation der Lösungen im politischen Entscheidungsprozess. Unser Ziel ist es, bestmögliche Lösungen zu präsentieren, die eine breite Akzeptanz finden.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr"/>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:philosophie:de0609d:editor</t>
         </is>
       </c>
     </row>
@@ -2120,18 +2120,18 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir denken Lösungen vom Ende her: strategische, technische, betriebs- und finanzwirtschaftliche, juristische und steuerliche Lösungen stellen wir dafür in den Gesamtkontext.&lt;/p&gt;</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr"/>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.0.elements.0.elements.2.settings.editor</t>
+          <t>live:leistungen:384d4e7:title</t>
         </is>
       </c>
     </row>
@@ -2148,13 +2148,13 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Unser Anspruch</t>
+          <t>Interdisziplinäre&lt;br&gt;&lt;span class="text-bg-green"&gt;Beratung.&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr"/>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.1.elements.0.elements.0.settings.title</t>
+          <t>live:leistungen:f80ec52:title</t>
         </is>
       </c>
     </row>
@@ -2166,18 +2166,18 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Experten für Ihre Beratung.</t>
+          <t>&lt;p&gt;Wir denken Lösungen vom Ende her: strategische, technische, betriebs- und finanzwirtschaftliche, juristische und steuerliche Lösungen stellen wir dafür in den Gesamtkontext.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr"/>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.1.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:df2021c:editor</t>
         </is>
       </c>
     </row>
@@ -2189,18 +2189,18 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Die Energiesozietät ist seit ihrer Gründung Ende 2023 dynamisch gewachsen und verfügt heute über ein Team mit großem Erfahrungsschatz. Viele Teammitglieder haben jahrelang erfolgreich in Big-Four-Gesellschaften, spezialisierten Beratungsgesellschaften und Kanzleien gearbeitet.&lt;/p&gt;</t>
+          <t>Unser Anspruch</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr"/>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.1.elements.1.elements.0.settings.editor</t>
+          <t>live:leistungen:cc808f7:title</t>
         </is>
       </c>
     </row>
@@ -2212,209 +2212,209 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Sollten wir selbst einmal nicht die geeigneten Spezialisten im Team haben, um Ihre Fragen bestmöglich zu beantworten, kooperieren wir mit namhaften Beratungsgesellschaften, mit denen wir seit vielen Jahren vertrauensvoll zusammenarbeiten.&lt;/p&gt;</t>
+          <t>Experten für Ihre Beratung.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr"/>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>leistungen.elementor.1.elements.1.elements.1.settings.editor</t>
+          <t>live:leistungen:fcd8206:title</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>&lt;p&gt;Unseren Mandanten ist eines gemein: Sie bewegen sich alle in einem hochkomplexen und sich kontinuierlich weiterentwickelnden Umfeld. Der politische Rahmen, regulatorische Anforderungen und technisch-wirtschaftliche Lösungsoptionen verändern sich fortwährend. Entscheidungsträger sind gefordert, in diesem dynamischen Umfeld gute Entscheidungen zu treffen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr"/>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.title</t>
+          <t>live:leistungen:6ff32c6:editor</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>01 · Rechtsberatung</t>
+          <t>&lt;p&gt;Die Energiesozietät ist seit ihrer Gründung Ende 2023 dynamisch gewachsen und verfügt heute über ein Team mit großem Erfahrungsschatz. Viele Teammitglieder haben jahrelang erfolgreich in Big-Four-Gesellschaften, spezialisierten Beratungsgesellschaften und Kanzleien gearbeitet.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr"/>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:b34aeee:editor</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Wir stellen juristische Lösungen in den Gesamtkontext — mit Blick auf das wirtschaftliche Ziel.</t>
+          <t>&lt;p&gt;Sollten wir selbst einmal nicht die geeigneten Spezialisten im Team haben, um Ihre Fragen bestmöglich zu beantworten, kooperieren wir mit namhaften Beratungsgesellschaften, mit denen wir seit vielen Jahren vertrauensvoll zusammenarbeiten.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr"/>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.0.elements.0.elements.2.settings.title</t>
+          <t>live:leistungen:58e656d:editor</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir stellen juristische Lösungen in den Gesamtkontext. Mit einem ausgeprägten Verständnis von Energiemärkten, Verwaltungsorganisationen und politischen Entscheidungsprozessen.&lt;/p&gt;</t>
+          <t>&lt;span class="es-bereich__num"&gt;01 / 03&lt;/span&gt;&lt;span class="es-bereich__sep"&gt;&lt;/span&gt;&lt;span class="es-bereich__sub"&gt;Juristische Lösungen im Gesamtkontext&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr"/>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.0.elements.0.elements.3.settings.editor</t>
+          <t>live:leistungen:7e7d8e3:title</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
+          <t>Leistungen</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
           <t>Rechtsberatung</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>Überschrift</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Was wir für Sie tun</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr"/>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:leistungen:eaa52c7:title</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Wir stellen juristische Lösungen in den Gesamtkontext — mit Blick auf das wirtschaftliche Ziel.</t>
+          <t>&lt;p&gt;Wir stellen juristische Lösungen in den Gesamtkontext.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr"/>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:40c1aee:editor</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Button/Text</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir haben ein ausgeprägtes Verständnis von Energiemärkten, Verwaltungsorganisationen und ihren politischen Entscheidungsprozessen. Politikberatung ist integraler Bestandteil unserer Tätigkeit, um die Projekte unserer Mandanten zum Erfolg zu führen.&lt;/p&gt;</t>
+          <t>Zur Rechtsberatung →</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr"/>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.2.elements.0.elements.2.settings.editor</t>
+          <t>live:leistungen:db95671:text</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Energiewirtschaftsrechtliche Fragestellungen stehen selten für sich allein — sie sind eingebettet in unternehmerische, steuerliche und regulatorische Zusammenhänge. Wir beraten interdisziplinär, Hand in Hand mit unseren Steuer- und Unternehmensberatern.&lt;/p&gt;</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr"/>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.2.elements.0.elements.3.settings.editor</t>
+          <t>live:leistungen:edd4fe8:title</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -2424,20 +2424,20 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Beratungsfelder</t>
+          <t>&lt;span class="es-bereich__num"&gt;02 / 03&lt;/span&gt;&lt;span class="es-bereich__sep"&gt;&lt;/span&gt;&lt;span class="es-bereich__sub"&gt;Fortlaufend · Gestaltend · Strukturierend&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr"/>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.2.elements.1.elements.0.settings.title</t>
+          <t>live:leistungen:8ce8498:title</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -2447,66 +2447,66 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Aus diesem Feld</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr"/>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.3.elements.0.elements.0.settings.title</t>
+          <t>live:leistungen:877be17:title</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Rechtsberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Publikationen &amp; Fachbeiträge</t>
+          <t>&lt;p&gt;Fortlaufende Steuerberatung, Gestaltungsberatung oder herausfordernde Neustrukturierungen?&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr"/>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>rechtsberatung.elementor.3.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:f606c90:editor</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Button/Text</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Zur Steuerberatung →</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr"/>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.title</t>
+          <t>live:leistungen:dd7d1ec:text</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
@@ -2516,20 +2516,20 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>02 · Steuerberatung</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr"/>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:c181737:title</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
@@ -2539,112 +2539,112 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Besonderes Know-how in der Betreuung der öffentlichen Hand — erfolgreich eingesetzt auch in der Privatwirtschaft.</t>
+          <t>&lt;span class="es-bereich__num"&gt;03 / 03&lt;/span&gt;&lt;span class="es-bereich__sep"&gt;&lt;/span&gt;&lt;span class="es-bereich__sub"&gt;Strategie · Wirtschaft · Finanzen&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr"/>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.0.elements.0.elements.2.settings.title</t>
+          <t>live:leistungen:9152915:title</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Fortlaufende Steuerberatung, Gestaltungsberatung oder herausfordernde Neustrukturierungen — mit besonderem Know-how in der Betreuung der öffentlichen Hand und ihrer Unternehmen.&lt;/p&gt;</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr"/>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.0.elements.0.elements.3.settings.editor</t>
+          <t>live:leistungen:07b85ef:title</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Was wir für Sie tun</t>
+          <t>&lt;p&gt;Wir navigieren Sie durch die Anforderungen neuer Energieträger und -erzeugungsarten sowie ihrer wirtschaftlichen und finanziellen Fragestellungen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr"/>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:leistungen:ec7789f:editor</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Button/Text</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Besonderes Know-how in der Betreuung der öffentlichen Hand — erfolgreich eingesetzt auch in der Privatwirtschaft.</t>
+          <t>Zur Unternehmensberatung →</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr"/>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:leistungen:ec9dff6:text</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Leistungen</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir kennen die steuerlichen Besonderheiten von Eigenbetrieben, Beteiligungsgesellschaften und juristischen Personen des öffentlichen Rechts. Dieses Wissen setzen wir ebenso erfolgreich in der Privatwirtschaft ein.&lt;/p&gt;</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr"/>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.2.elements.0.elements.2.settings.editor</t>
+          <t>live:leistungen:d86d7a3:title</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -2654,20 +2654,20 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Von der laufenden Steuerberatung über Deklarationen bis hin zu strukturellen Neustrukturierungen — wir denken steuerliche Lösungen im Gesamtkontext unserer Mandanten.&lt;/p&gt;</t>
+          <t>&lt;div class="es-article__crumb" style="margin-bottom:28px;"&gt;&lt;a href="/leistungen/" style="color:inherit;"&gt;Leistungen&lt;/a&gt;  /  Rechtsberatung&lt;/div&gt;</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr"/>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.2.elements.0.elements.3.settings.editor</t>
+          <t>live:rechtsberatung:61e00bd:editor</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -2677,20 +2677,20 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Beratungsfelder</t>
+          <t>01 · Rechtsberatung</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr"/>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.2.elements.1.elements.0.settings.title</t>
+          <t>live:rechtsberatung:d9d4dc0:title</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -2700,66 +2700,66 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Aus diesem Feld</t>
+          <t>Wir stellen juristische Lösungen in den Gesamtkontext.</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr"/>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.3.elements.0.elements.0.settings.title</t>
+          <t>live:rechtsberatung:b7d4c1c:title</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Steuerberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Publikationen &amp; Fachbeiträge</t>
+          <t>&lt;p&gt;Wir haben ein ausgeprägtes Verständnis von Energiemärkten, Verwaltungsorganisationen und ihren politischen Entscheidungsprozessen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr"/>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>steuerberatung.elementor.3.elements.0.elements.1.settings.title</t>
+          <t>live:rechtsberatung:8620aef:editor</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Was wir für Sie tun</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr"/>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.title</t>
+          <t>live:rechtsberatung:306958d:title</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -2769,43 +2769,43 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>03 · Unternehmensberatung</t>
+          <t>Rechtsberatung.</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr"/>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:rechtsberatung:e71d1f5:title</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Investier- und Finanzierbarkeit von Transformation erreichen.</t>
+          <t>&lt;p&gt;Mit unserem Beratungsangebot adressieren wir Energieversorgungsunternehmen, Bund, Länder und Kommunen sowie deren Einrichtungen und Unternehmen sowie private und öffentliche Infrastrukturdienstleister und Investoren.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr"/>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.0.elements.0.elements.2.settings.title</t>
+          <t>live:rechtsberatung:83ef114:editor</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -2815,20 +2815,20 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Wir navigieren Sie durch die Anforderungen neuer Energieträger und Erzeugungsarten sowie die damit verbundenen wirtschaftlichen und finanziellen Fragestellungen.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Wir haben ein ausgeprägtes Verständnis von Energiemärkten, Verwaltungsorganisationen und ihren politischen Entscheidungsprozessen. Politikberatung ist integraler Bestandteil unserer Tätigkeit, um Ihre Projekte zum Erfolg zu führen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr"/>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.0.elements.0.elements.3.settings.editor</t>
+          <t>live:rechtsberatung:ebe46a9:editor</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -2838,20 +2838,20 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Was wir für Sie tun</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr"/>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:rechtsberatung:6a126bf:title</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -2861,43 +2861,43 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Investier- und Finanzierbarkeit von Transformation erreichen.</t>
+          <t>Aus diesem Feld</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr"/>
       <c r="E98" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:rechtsberatung:09c4bc9:title</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;In der Energiebranche erzeugt die Erfordernis, den Klimazielen gerecht zu werden, enormen Druck. Traditionellen Geschäftsmodellen werden Grenzen aufgezeigt. Neue Energieträger, innovative Erzeugungstechnologien und leistungsfähige Netze sollen die Energieversorgung von morgen sicherstellen.&lt;/p&gt;</t>
+          <t>Publikationen &amp; Fachbeiträge</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr"/>
       <c r="E99" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.2.elements.0.elements.2.settings.editor</t>
+          <t>live:rechtsberatung:67bd19a:title</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Rechtsberatung</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
@@ -2907,43 +2907,43 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Unsere Experten begleiten Sie von Beginn an — als Sparringspartner, bei der Entwicklung von Strategieoptionen, deren Konkretisierung in Business Plänen, bei der Finanzierung und der Suche nach strategischen Partnern für die Umsetzung.&lt;/p&gt;</t>
+          <t>&lt;p style="margin-top:32px;"&gt;&lt;a class="es-link" href="/publikationen/?feld=rechtsberatung"&gt;Alle Publikationen →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr"/>
       <c r="E100" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.2.elements.0.elements.3.settings.editor</t>
+          <t>live:rechtsberatung:444e298:editor</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Beratungsfelder</t>
+          <t>&lt;div class="es-article__crumb" style="margin-bottom:28px;"&gt;&lt;a href="/leistungen/" style="color:inherit;"&gt;Leistungen&lt;/a&gt;  /  Steuerberatung&lt;/div&gt;</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr"/>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.2.elements.1.elements.0.settings.title</t>
+          <t>live:steuerberatung:e473fe5:editor</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
@@ -2953,20 +2953,20 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Aus diesem Feld</t>
+          <t>02 · Steuerberatung</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr"/>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.3.elements.0.elements.0.settings.title</t>
+          <t>live:steuerberatung:25c68b2:title</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Unternehmensberatung</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
@@ -2976,43 +2976,43 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Publikationen &amp; Fachbeiträge</t>
+          <t>Fortlaufende Steuerberatung, Gestaltungsberatung oder herausfordernde Neustrukturierungen?</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr"/>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>unternehmensberatung.elementor.3.elements.0.elements.1.settings.title</t>
+          <t>live:steuerberatung:efa3375:title</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>&lt;p&gt;Wir begleiten unsere Mandanten umfassend bei allen steuerlichen Fragen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr"/>
       <c r="E104" s="6" t="inlineStr">
         <is>
-          <t>team.title</t>
+          <t>live:steuerberatung:5b585ea:editor</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
@@ -3022,20 +3022,20 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Was wir für Sie tun</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr"/>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:steuerberatung:7338749:title</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -3045,20 +3045,20 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Beratung mit&lt;br&gt;Gesicht.</t>
+          <t>Steuerberatung.</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr"/>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:steuerberatung:06d871d:title</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -3068,43 +3068,43 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;In der Energiesozietät hat jahrzehntelange Erfahrung einen agilen und pragmatischen Rahmen bekommen.&lt;/p&gt;</t>
+          <t>&lt;p&gt;Wir begleiten unsere Mandanten umfassend bei allen steuerlichen Fragen: Unternehmen der Privat- und Kommunalwirtschaft, juristische Personen des öffentlichen Rechts, Privatpersonen und Existenzgründer.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr"/>
       <c r="E107" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.0.elements.0.elements.2.settings.editor</t>
+          <t>live:steuerberatung:c078e0e:editor</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Netzwerk</t>
+          <t>&lt;p&gt;Besonderes Know-how haben wir in der Betreuung der öffentlichen Hand und ihrer Unternehmen – dieses Wissen setzen wir ebenso erfolgreich in der Privatwirtschaft ein.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr"/>
       <c r="E108" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:steuerberatung:a0fe563:editor</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
@@ -3114,181 +3114,181 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Kooperationen mit namhaften Beratungshäusern.</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr"/>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:steuerberatung:c9d87c4:title</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Sollten wir selbst einmal nicht die geeigneten Spezialisten im Team haben, kooperieren wir mit namhaften Beratungsgesellschaften, mit denen wir seit vielen Jahren vertrauensvoll zusammenarbeiten. Sprechen Sie uns gerne direkt an.&lt;/p&gt;</t>
+          <t>Aus diesem Feld</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr"/>
       <c r="E110" s="6" t="inlineStr">
         <is>
-          <t>team.elementor.2.elements.1.elements.0.settings.editor</t>
+          <t>live:steuerberatung:7d96f28:title</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>Publikationen &amp; Fachbeiträge</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr"/>
       <c r="E111" s="6" t="inlineStr">
         <is>
-          <t>publikationen.title</t>
+          <t>live:steuerberatung:507e86f:title</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>Steuerberatung</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>&lt;p style="margin-top:32px;"&gt;&lt;a class="es-link" href="/publikationen/?feld=steuerberatung"&gt;Alle Publikationen →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr"/>
       <c r="E112" s="6" t="inlineStr">
         <is>
-          <t>publikationen.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:steuerberatung:2572317:editor</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>Bücher,&lt;br&gt;Kommentare&lt;br&gt;&lt;span style="color:rgba(255,255,255,0.55);"&gt;&amp;amp; Fachaufsätze.&lt;/span&gt;</t>
+          <t>&lt;div class="es-article__crumb" style="margin-bottom:28px;"&gt;&lt;a href="/leistungen/" style="color:inherit;"&gt;Leistungen&lt;/a&gt;  /  Unternehmensberatung&lt;/div&gt;</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr"/>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>publikationen.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:unternehmensberatung:9a1588a:editor</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Publikationen</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Unser Team veröffentlicht regelmäßig in Fachzeitschriften, Kommentaren und Handbüchern zum Energiewirtschafts-, Vergabe-, Kommunal- und Steuerrecht. Eine Auswahl aus den letzten Jahren.&lt;/p&gt;</t>
+          <t>03 · Unternehmensberatung</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr"/>
       <c r="E114" s="6" t="inlineStr">
         <is>
-          <t>publikationen.elementor.0.elements.0.elements.2.settings.editor</t>
+          <t>live:unternehmensberatung:0dbc0c3:title</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Wir navigieren Sie durch die Anforderungen neuer Energieträger und Erzeugungsarten sowie ihrer wirtschaftlichen und finanziellen Fragestellungen.</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr"/>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>karriere.title</t>
+          <t>live:unternehmensberatung:3ddb6e0:title</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>&lt;p&gt;In der Energiebranche erzeugt das Erfordernis, den Klimazielen gerecht zu werden, einen enormen Druck – traditionellen Geschäftsmodellen werden Grenzen aufgezeigt.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr"/>
       <c r="E116" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:unternehmensberatung:02c1e33:editor</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -3298,112 +3298,112 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Starte gemeinsam&lt;br&gt;mit uns &lt;span class="text-bg-green"&gt;durch.&lt;/span&gt;</t>
+          <t>Was wir für Sie tun</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr"/>
       <c r="E117" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:unternehmensberatung:ddae754:title</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;Entfalte Dich selbst in einem jungen, schnell wachsenden Beratungsunternehmen. Wir suchen Persönlichkeiten, die Verantwortung übernehmen wollen.&lt;/p&gt;</t>
+          <t>Unternehmensberatung.</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr"/>
       <c r="E118" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.0.elements.1.elements.0.settings.editor</t>
+          <t>live:unternehmensberatung:46065bc:title</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Offene Positionen</t>
+          <t>&lt;p&gt;&lt;span style="color: inherit;"&gt;Neue Energieträger, innovative Erzeugungstechnologien und leistungsfähige Netze sollen die Energieversorgung von Morgen nachhaltig gestalten. Für Unternehmen der Energiewirtschaft ergeben sich daraus erhebliche Herausforderungen: Mengen und Margen im Bestandsgeschäft sichern, neue Geschäftsmodelle entwickeln, die Unternehmensorganisationen für diese Aufgaben befähigen und die Finanzierungs- und damit die Investitionsfähigkeit erhalten. &lt;/span&gt;&lt;/p&gt;&lt;p&gt; &lt;/p&gt;</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr"/>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.1.elements.0.elements.0.settings.title</t>
+          <t>live:unternehmensberatung:3df265d:editor</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Warum wir</t>
+          <t>&lt;p&gt;&lt;span style="color: inherit;"&gt;Wir beraten Unternehmen, Kommunen und Investoren &lt;/span&gt;bei diesen herausfordernden Fragestellungen von Beginn an: als Sparringspartner in allerersten Überlegungen, bei der Entwicklung von Strategie- und Modelloptionen, der regulatorischen Optimierung, bei deren Konkretisierung und Überprüfung in Business Plänen, bei der Optimierung der Kapitalstruktur und der Finanzierung sowie bei der Suche nach strategischen Partnern für die Umsetzung.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr"/>
       <c r="E120" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.2.elements.0.elements.0.settings.title</t>
+          <t>live:unternehmensberatung:9ef1268:editor</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Was Dich bei uns erwartet.</t>
+          <t>&lt;p&gt;&lt;span style="font-size: inherit; color: inherit;"&gt;Unsere Stärke &lt;/span&gt;&lt;span style="font-size: inherit; color: inherit;"&gt;liegt in der Übersetzung strategischer Zielbilder &lt;/span&gt;&lt;span style="font-size: inherit; color: inherit;"&gt;in wirtschaftlich tragfähige Entscheidungen, Strukturen und Umsetzungsprogramme, &lt;/span&gt;&lt;span style="font-size: inherit; color: inherit;"&gt;innerhalb von Kommunen und Versorgungsunternehmen. Unser Beratung ist erfolgreich, wenn wir für ihre Herausforderungen tragefähige Lösungen entwickeln, die auf eine breite politische Zustimmung stößt.&lt;/span&gt;&lt;/p&gt;&lt;p&gt; &lt;/p&gt;</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr"/>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.2.elements.0.elements.1.settings.title</t>
+          <t>live:unternehmensberatung:9abba1a:editor</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -3413,43 +3413,43 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Echte Verantwortung</t>
+          <t>Beratungsfelder</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr"/>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.0.elements.1.settings.title</t>
+          <t>live:unternehmensberatung:06f6a7c:title</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Du arbeitest von Tag eins direkt am Mandat, mit Mandantenkontakt und eigener Themenverantwortung.</t>
+          <t>Aus diesem Feld</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr"/>
       <c r="E123" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.0.elements.2.settings.editor</t>
+          <t>live:unternehmensberatung:34fe075:title</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -3459,20 +3459,20 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Interdisziplinarität</t>
+          <t>Publikationen &amp;amp; Fachbeiträge</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr"/>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.1.elements.1.settings.title</t>
+          <t>live:unternehmensberatung:aac8ab4:title</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Unternehmensberatung</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -3482,20 +3482,20 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Kein Silodenken. Wir bringen Recht, Steuern und Unternehmensberatung zusammen — und Dich mittendrin.</t>
+          <t>&lt;p style="margin-top:32px;"&gt;&lt;a class="es-link" href="/publikationen/?feld=unternehmensberatung"&gt;Alle Publikationen →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr"/>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.1.elements.2.settings.editor</t>
+          <t>live:unternehmensberatung:2d98bb7:editor</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -3505,66 +3505,66 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Persönliche Entwicklung</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr"/>
       <c r="E126" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.2.elements.1.settings.title</t>
+          <t>live:team:24a78db:title</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>Karriere</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Absatz</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Fortbildung, Promotion, Fachanwaltschaften — wir fördern gezielt und individuell.</t>
+          <t>Vielleicht kennen&lt;br&gt;Sie uns &lt;span class="text-bg-green"&gt;schon?&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr"/>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>karriere.elementor.3.elements.2.elements.2.settings.editor</t>
+          <t>live:team:fefc70e:title</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>&lt;p&gt;Die Energiesozietät gibt einem sehr erfahrenen Team einen agilen und pragmatischen Rahmen. Die Teammitglieder arbeiten seit vielen Jahren zusammen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr"/>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>news.title</t>
+          <t>live:team:9616110:editor</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -3574,20 +3574,20 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Netzwerk</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr"/>
       <c r="E129" s="6" t="inlineStr">
         <is>
-          <t>news.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:team:1087ce4:title</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>News</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -3597,66 +3597,66 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Aus der&lt;br&gt;&lt;span class="text-bg-green"&gt;Energiebranche.&lt;/span&gt;</t>
+          <t>Kooperationen mit namhaften Beratungshäusern.</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr"/>
       <c r="E130" s="6" t="inlineStr">
         <is>
-          <t>news.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:team:4493ccd:title</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>Veranstaltungen</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Veranstaltungen</t>
+          <t>&lt;p&gt;Wir sind seit vielen Jahren verlässliche Berater für die Kommunalwirtschaft, Länder, Bund und private Unternehmen. Wir freuen uns auf ein kontinuierlich wachsendes Team, um Ihre Fragestellungen interdisziplinär und ganzheitlich betrachten zu können.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr"/>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>veranstaltungen.title</t>
+          <t>live:team:9d0744e:editor</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>Veranstaltungen</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Veranstaltungen</t>
+          <t>&lt;p&gt;Sollten wir selbst einmal nicht die geeigneten Spezialisten im Team haben, kooperieren wir mit namhaften Beratungsgesellschaften, mit denen wir seit vielen Jahren vertrauensvoll zusammenarbeiten. Sprechen Sie uns gerne direkt an.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr"/>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>veranstaltungen.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:team:bde259f:editor</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>Veranstaltungen</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -3666,66 +3666,66 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Wo wir&lt;br&gt;sprechen.</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr"/>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>veranstaltungen.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:karriere:cb9ef8f:title</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Starte gemeinsam&lt;br&gt;mit uns &lt;span class="text-bg-green"&gt;durch!&lt;/span&gt;</t>
         </is>
       </c>
       <c r="D134" s="5" t="inlineStr"/>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>kontakt.title</t>
+          <t>live:karriere:5ff49d7:title</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>&lt;p&gt;Entfalte Dich selbst in einem jungen, schnell wachsenden Beratungsunternehmen.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr"/>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>kontakt.elementor.0.elements.0.elements.0.settings.title</t>
+          <t>live:karriere:5359b87:editor</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -3735,43 +3735,43 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Sprechen Sie&lt;br&gt;mit uns.</t>
+          <t>Offene Positionen</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr"/>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>kontakt.elementor.0.elements.0.elements.1.settings.title</t>
+          <t>live:karriere:70d71ea:title</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Überschrift</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Schreiben Sie uns</t>
+          <t>&lt;p style="margin-top:32px;"&gt;&lt;a class="es-link" href="mailto:info@energiesozietaet.de?subject=Initiativbewerbung"&gt;Initiativbewerbung →&lt;/a&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr"/>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>kontakt.elementor.1.elements.0.elements.0.settings.title</t>
+          <t>live:karriere:e29a862:editor</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -3781,20 +3781,20 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Wir antworten innerhalb eines Werktags.</t>
+          <t>Warum wir</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr"/>
       <c r="E138" s="6" t="inlineStr">
         <is>
-          <t>kontakt.elementor.1.elements.0.elements.1.settings.title</t>
+          <t>live:karriere:6fa317d:title</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>Kontakt</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -3804,59 +3804,565 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Unsere Standorte</t>
+          <t>Was Dich bei uns erwartet.</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr"/>
       <c r="E139" s="6" t="inlineStr">
         <is>
-          <t>kontakt.elementor.1.elements.1.elements.0.settings.title</t>
+          <t>live:karriere:f4b5ed6:title</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>Impressum</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Überschrift</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Impressum</t>
+          <t>Echte Verantwortung</t>
         </is>
       </c>
       <c r="D140" s="5" t="inlineStr"/>
       <c r="E140" s="6" t="inlineStr">
         <is>
-          <t>impressum.title</t>
+          <t>live:karriere:03225be:title</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>Datenschutzerklärung</t>
+          <t>Karriere</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Seitentitel</t>
+          <t>Absatz</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Datenschutzerklärung</t>
+          <t>&lt;p&gt;Du arbeitest von Tag eins direkt am Mandat, mit Mandantenkontakt und eigener Themenverantwortung.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr"/>
       <c r="E141" s="6" t="inlineStr">
         <is>
-          <t>datenschutzerklaerung.title</t>
+          <t>live:karriere:070ba97:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>Karriere</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>Interdisziplinarität</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr"/>
+      <c r="E142" s="6" t="inlineStr">
+        <is>
+          <t>live:karriere:66ff972:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>Karriere</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Kein Silodenken. Wir bringen Recht, Steuern und Unternehmensberatung zusammen – und Dich mittendrin.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr"/>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
+          <t>live:karriere:8a124db:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="4" t="inlineStr">
+        <is>
+          <t>Karriere</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>Persönliche Entwicklung</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr"/>
+      <c r="E144" s="6" t="inlineStr">
+        <is>
+          <t>live:karriere:befaa3d:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>Karriere</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Fortbildung, Promotion, Fachanwaltschaften – wir fördern gezielt und individuell.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr"/>
+      <c r="E145" s="6" t="inlineStr">
+        <is>
+          <t>live:karriere:c6f02b4:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr"/>
+      <c r="E146" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:3100e45:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>Wir freuen uns auf Ihre&lt;br&gt;&lt;span class="text-bg-green"&gt;Kontaktaufnahme.&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr"/>
+      <c r="E147" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:cfc62f7:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Bitte zögern Sie nicht, uns anzusprechen.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr"/>
+      <c r="E148" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:45f87a7:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>Schreiben Sie uns</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr"/>
+      <c r="E149" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:bf53f63:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>Kontaktformular</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr"/>
+      <c r="E150" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:d7a6dff:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Sie haben ein konkretes Anliegen oder wissen schon, mit wem Sie bei der Energiesozietät sprechen möchten? Dann nutzen Sie gerne in der Rubrik &lt;a href="/team/"&gt;Team&lt;/a&gt; die Möglichkeit zur direkten Kontaktaufnahme mit dem jeweiligen Experten.&lt;/p&gt;&lt;p&gt;Sie möchten uns kennenlernen? Dann hinterlassen Sie uns gerne eine Nachricht mit Ihren Kontaktdaten. Wir melden uns umgehend bei Ihnen, um einen Termin zu vereinbaren.&lt;/p&gt;&lt;p&gt;Sie wünschen eine Einladung zu einem Event oder sind an Publikationen interessiert? Lassen Sie es uns bitte wissen.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr"/>
+      <c r="E151" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:329ef85:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>Kontakt</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="inlineStr">
+        <is>
+          <t>Unsere Büros</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr"/>
+      <c r="E152" s="6" t="inlineStr">
+        <is>
+          <t>live:kontakt:7494226:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr"/>
+      <c r="E153" s="6" t="inlineStr">
+        <is>
+          <t>live:news:9e88215:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="inlineStr">
+        <is>
+          <t>Aktuelles aus&lt;br&gt;der &lt;span class="text-bg-green"&gt;Kanzlei.&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr"/>
+      <c r="E154" s="6" t="inlineStr">
+        <is>
+          <t>live:news:b4d89f9:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Unser Anspruch</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr"/>
+      <c r="E155" s="6" t="inlineStr">
+        <is>
+          <t>live:news:6a164f9:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>„Wir möchten unsere Mandanten mit exzellenten, pragmatischen Lösungen unterstützen."</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr"/>
+      <c r="E156" s="6" t="inlineStr">
+        <is>
+          <t>live:news:d6ec803:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p class="es-gf-quote__name"&gt;Prof. Dr. Sven-Joachim Otto&lt;/p&gt;&lt;p class="es-gf-quote__role"&gt;Partner&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr"/>
+      <c r="E157" s="6" t="inlineStr">
+        <is>
+          <t>live:news:439c91c:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>Veranstaltungen</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C158" s="4" t="inlineStr">
+        <is>
+          <t>Veranstaltungen</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr"/>
+      <c r="E158" s="6" t="inlineStr">
+        <is>
+          <t>live:veranstaltungen:b6b6c3c:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>Veranstaltungen</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Aktuelle&lt;br&gt;&lt;span class="text-bg-green"&gt;Termine.&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr"/>
+      <c r="E159" s="6" t="inlineStr">
+        <is>
+          <t>live:veranstaltungen:9a3aa4f:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>Publikationen</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>Publikationen</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr"/>
+      <c r="E160" s="6" t="inlineStr">
+        <is>
+          <t>live:publikationen:66ce230:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>Publikationen</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>Überschrift</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>Unsere&lt;br&gt;&lt;span class="text-bg-green"&gt;Veröffentlichungen.&lt;/span&gt;</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr"/>
+      <c r="E161" s="6" t="inlineStr">
+        <is>
+          <t>live:publikationen:5c75ea7:title</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>Publikationen</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Energie- und Kommunalwirtschaft befinden sich in einem fortwährenden Wandel. Deswegen lernen wir ständig hinzu. Manche unserer neuen Erkenntnisse lohnt es sich zu teilen.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr"/>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>live:publikationen:a159fa4:editor</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>Publikationen</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>Absatz</t>
+        </is>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Die Herausforderungen unserer Mandanten, die Transformation der öffentlichen Hand und der Energiewirtschaft voranzutreiben, stellen uns tagtäglich vor neue Herausforderungen. Lösungen für die Fragen unserer Zeit zu finden, erfordert es, sich auf seine Erfahrungen und Kompetenzen zu verlassen und erlernte Methoden in neuen Aufgabenstellungen anzuwenden. Gleichzeitig verändert sich der Handlungsrahmen, in dem wir uns bewegen, fortwährend.&lt;/p&gt;&lt;p&gt;Es gibt also zahlreiche Anlässe, Wissen und Sichtweisen zu teilen, um am Puls der Zeit zu sein.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr"/>
+      <c r="E163" s="6" t="inlineStr">
+        <is>
+          <t>live:publikationen:03d4032:editor</t>
         </is>
       </c>
     </row>

</xml_diff>